<commit_message>
Added some hidden parameter groups, and also added param clamping for various parameters
to prevent improper entry.
</commit_message>
<xml_diff>
--- a/xplorer-params-disposition-v1.xlsx
+++ b/xplorer-params-disposition-v1.xlsx
@@ -4557,7 +4557,7 @@
         <v>0</v>
       </c>
       <c r="E201" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="202">
@@ -5292,7 +5292,7 @@
         <v>0</v>
       </c>
       <c r="E236" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="237">

</xml_diff>